<commit_message>
WMS-024: feedback points implemented
</commit_message>
<xml_diff>
--- a/demo-assets/lonestar_sales_week38.xlsx
+++ b/demo-assets/lonestar_sales_week38.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A83162-D7EE-4808-93CE-076581D7F650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Registrations" state="visible" r:id="rId4"/>
+    <sheet name="Registrations" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -46,7 +50,7 @@
     <t>Invoice number</t>
   </si>
   <si>
-    <t>263510101</t>
+    <t>SC680-263510101</t>
   </si>
   <si>
     <t>2635-L01</t>
@@ -76,7 +80,7 @@
     <t>LS-38-1001</t>
   </si>
   <si>
-    <t>263510108</t>
+    <t>SC480-263510108</t>
   </si>
   <si>
     <t>2635-L02</t>
@@ -103,7 +107,7 @@
     <t>LS-38-1002</t>
   </si>
   <si>
-    <t>263510115</t>
+    <t>SC260-263510115</t>
   </si>
   <si>
     <t>2635-L03</t>
@@ -127,7 +131,7 @@
     <t>LS-38-1003</t>
   </si>
   <si>
-    <t>263510122</t>
+    <t>SM482V-263510122</t>
   </si>
   <si>
     <t>SM482V</t>
@@ -148,7 +152,7 @@
     <t>LS-38-1004</t>
   </si>
   <si>
-    <t>263510129</t>
+    <t>SM382V-263510129</t>
   </si>
   <si>
     <t>SM382V</t>
@@ -172,7 +176,7 @@
     <t>LS-38-1005</t>
   </si>
   <si>
-    <t>263510136</t>
+    <t>JL3KH6-263510136</t>
   </si>
   <si>
     <t>JL3KH6</t>
@@ -214,7 +218,7 @@
     <t>LS-38-1007</t>
   </si>
   <si>
-    <t>263510150</t>
+    <t>MR45-263510150</t>
   </si>
   <si>
     <t>MR45</t>
@@ -235,7 +239,7 @@
     <t>LS-38-1008</t>
   </si>
   <si>
-    <t>263510157</t>
+    <t>MG44-263510157</t>
   </si>
   <si>
     <t>MG44</t>
@@ -259,7 +263,7 @@
     <t>LS-38-1009</t>
   </si>
   <si>
-    <t>263510164</t>
+    <t>DR82-263510164</t>
   </si>
   <si>
     <t>DR82</t>
@@ -280,7 +284,7 @@
     <t>LS-38-1010</t>
   </si>
   <si>
-    <t>263510171</t>
+    <t>SRS1-263510171</t>
   </si>
   <si>
     <t>SRS1</t>
@@ -301,7 +305,7 @@
     <t>LS-38-1011</t>
   </si>
   <si>
-    <t>263510178</t>
+    <t>STA2-263510178</t>
   </si>
   <si>
     <t>STA2</t>
@@ -322,7 +326,7 @@
     <t>LS-38-1012</t>
   </si>
   <si>
-    <t>252811902</t>
+    <t>MG44-252811902</t>
   </si>
   <si>
     <t>Mike Delgado</t>
@@ -343,7 +347,7 @@
     <t>LS-38-1013</t>
   </si>
   <si>
-    <t>263510192</t>
+    <t>SC480-263510192</t>
   </si>
   <si>
     <t>(713) 555-0133</t>
@@ -352,7 +356,7 @@
     <t>LS-38-1014</t>
   </si>
   <si>
-    <t>263510199</t>
+    <t>SC260-263510199</t>
   </si>
   <si>
     <t>(713) 555-0134</t>
@@ -361,7 +365,7 @@
     <t>LS-38-1015</t>
   </si>
   <si>
-    <t>263510206</t>
+    <t>SM482V-263510206</t>
   </si>
   <si>
     <t>(713) 555-0135</t>
@@ -370,7 +374,7 @@
     <t>LS-38-1016</t>
   </si>
   <si>
-    <t>263510213</t>
+    <t>SM382V-263510213</t>
   </si>
   <si>
     <t>(713) 555-0136</t>
@@ -382,7 +386,7 @@
     <t>LS-38-1017</t>
   </si>
   <si>
-    <t>263510220</t>
+    <t>JL3KH6-263510220</t>
   </si>
   <si>
     <t>(713) 555-0137</t>
@@ -391,7 +395,7 @@
     <t>LS-38-1018</t>
   </si>
   <si>
-    <t>263510227</t>
+    <t>VP87-263510227</t>
   </si>
   <si>
     <t>VP87</t>
@@ -403,7 +407,7 @@
     <t>LS-38-1019</t>
   </si>
   <si>
-    <t>263510234</t>
+    <t>MR45-263510234</t>
   </si>
   <si>
     <t>(713) 555-0139</t>
@@ -412,7 +416,7 @@
     <t>LS-38-1020</t>
   </si>
   <si>
-    <t>263510241</t>
+    <t>MG44-263510241</t>
   </si>
   <si>
     <t>(713) 555-0140</t>
@@ -424,7 +428,7 @@
     <t>LS-38-1021</t>
   </si>
   <si>
-    <t>263510248</t>
+    <t>DR82-263510248</t>
   </si>
   <si>
     <t>(713) 555-0141</t>
@@ -433,7 +437,7 @@
     <t>LS-38-1022</t>
   </si>
   <si>
-    <t>263510255</t>
+    <t>SRS1-263510255</t>
   </si>
   <si>
     <t>(713) 555-0142</t>
@@ -442,7 +446,7 @@
     <t>LS-38-1023</t>
   </si>
   <si>
-    <t>263510262</t>
+    <t>STA2-263510262</t>
   </si>
   <si>
     <t>(713) 555-0143</t>
@@ -451,7 +455,7 @@
     <t>LS-38-1024</t>
   </si>
   <si>
-    <t>263510269</t>
+    <t>SC680-263510269</t>
   </si>
   <si>
     <t>(713) 555-0144</t>
@@ -466,20 +470,22 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -847,9 +853,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" style="1" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -905,7 +911,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="2">
-        <v>46279</v>
+        <v>44822</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
@@ -940,7 +946,7 @@
         <v>23</v>
       </c>
       <c r="D3" s="2">
-        <v>46280</v>
+        <v>46284</v>
       </c>
       <c r="E3" t="s">
         <v>24</v>
@@ -975,7 +981,7 @@
         <v>32</v>
       </c>
       <c r="D4" s="2">
-        <v>46281</v>
+        <v>46285</v>
       </c>
       <c r="E4" t="s">
         <v>33</v>
@@ -1010,7 +1016,7 @@
         <v>39</v>
       </c>
       <c r="D5" s="2">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="E5" t="s">
         <v>40</v>
@@ -1045,7 +1051,7 @@
         <v>46</v>
       </c>
       <c r="D6" s="2">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="E6" t="s">
         <v>47</v>
@@ -1080,7 +1086,7 @@
         <v>54</v>
       </c>
       <c r="D7" s="2">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="E7" t="s">
         <v>55</v>
@@ -1115,7 +1121,7 @@
         <v>61</v>
       </c>
       <c r="D8" s="2">
-        <v>46280</v>
+        <v>46284</v>
       </c>
       <c r="E8" t="s">
         <v>62</v>
@@ -1150,7 +1156,7 @@
         <v>68</v>
       </c>
       <c r="D9" s="2">
-        <v>46281</v>
+        <v>46285</v>
       </c>
       <c r="E9" t="s">
         <v>69</v>
@@ -1185,7 +1191,7 @@
         <v>75</v>
       </c>
       <c r="D10" s="2">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="E10" t="s">
         <v>76</v>
@@ -1220,7 +1226,7 @@
         <v>83</v>
       </c>
       <c r="D11" s="2">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="E11" t="s">
         <v>84</v>
@@ -1255,7 +1261,7 @@
         <v>90</v>
       </c>
       <c r="D12" s="2">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="E12" t="s">
         <v>91</v>
@@ -1290,7 +1296,7 @@
         <v>97</v>
       </c>
       <c r="D13" s="2">
-        <v>46280</v>
+        <v>45188</v>
       </c>
       <c r="E13" t="s">
         <v>98</v>
@@ -1322,10 +1328,10 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="D14" s="2">
-        <v>46281</v>
+        <v>46285</v>
       </c>
       <c r="E14" t="s">
         <v>104</v>
@@ -1360,7 +1366,7 @@
         <v>23</v>
       </c>
       <c r="D15" s="2">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -1395,7 +1401,7 @@
         <v>32</v>
       </c>
       <c r="D16" s="2">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
@@ -1430,7 +1436,7 @@
         <v>39</v>
       </c>
       <c r="D17" s="2">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="E17" t="s">
         <v>33</v>
@@ -1465,7 +1471,7 @@
         <v>46</v>
       </c>
       <c r="D18" s="2">
-        <v>46280</v>
+        <v>46284</v>
       </c>
       <c r="E18" t="s">
         <v>40</v>
@@ -1500,7 +1506,7 @@
         <v>54</v>
       </c>
       <c r="D19" s="2">
-        <v>46281</v>
+        <v>45555</v>
       </c>
       <c r="E19" t="s">
         <v>47</v>
@@ -1534,7 +1540,6 @@
       <c r="C20" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="2"/>
       <c r="E20" t="s">
         <v>55</v>
       </c>
@@ -1568,7 +1573,7 @@
         <v>68</v>
       </c>
       <c r="D21" s="2">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="E21" t="s">
         <v>62</v>
@@ -1603,7 +1608,7 @@
         <v>75</v>
       </c>
       <c r="D22" s="2">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="E22" t="s">
         <v>69</v>
@@ -1638,7 +1643,7 @@
         <v>83</v>
       </c>
       <c r="D23" s="2">
-        <v>46280</v>
+        <v>46284</v>
       </c>
       <c r="E23" t="s">
         <v>76</v>
@@ -1673,7 +1678,7 @@
         <v>90</v>
       </c>
       <c r="D24" s="2">
-        <v>46281</v>
+        <v>46285</v>
       </c>
       <c r="E24" t="s">
         <v>84</v>
@@ -1708,7 +1713,7 @@
         <v>97</v>
       </c>
       <c r="D25" s="2">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="E25" t="s">
         <v>91</v>
@@ -1743,7 +1748,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="2">
-        <v>46283</v>
+        <v>45922</v>
       </c>
       <c r="E26" t="s">
         <v>98</v>
@@ -1769,6 +1774,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>